<commit_message>
Populate MITRE ATT&CK technique column in Draft methodology workbooks.
Fill column J using ATT&CK v19.1-aligned technique IDs and names for AD, Azure, and WinBuild checks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Draft_AD_Methodology_FINAL.xlsx
+++ b/Draft_AD_Methodology_FINAL.xlsx
@@ -676,7 +676,12 @@
         </s:is>
       </s:c>
       <s:c r="I3" s="3" t="n"/>
-      <s:c r="J3" s="3" t="n"/>
+      <s:c r="J3" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1046 - Network Service Discovery
+T1595.002 - Vulnerability Scanning</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K3" s="3" t="n"/>
       <s:c r="L3" s="3" t="n"/>
       <s:c r="M3" s="3" t="n"/>
@@ -719,7 +724,12 @@
         </s:is>
       </s:c>
       <s:c r="I4" s="3" t="n"/>
-      <s:c r="J4" s="3" t="n"/>
+      <s:c r="J4" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1046 - Network Service Discovery
+T1595.002 - Vulnerability Scanning</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K4" s="3" t="n"/>
       <s:c r="L4" s="3" t="n"/>
       <s:c r="M4" s="3" t="n"/>
@@ -762,7 +772,12 @@
         </s:is>
       </s:c>
       <s:c r="I5" s="3" t="n"/>
-      <s:c r="J5" s="3" t="n"/>
+      <s:c r="J5" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1046 - Network Service Discovery
+T1595.002 - Vulnerability Scanning</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K5" s="3" t="n"/>
       <s:c r="L5" s="3" t="n"/>
       <s:c r="M5" s="3" t="n"/>
@@ -805,7 +820,13 @@
         </s:is>
       </s:c>
       <s:c r="I6" s="3" t="n"/>
-      <s:c r="J6" s="3" t="n"/>
+      <s:c r="J6" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1046 - Network Service Discovery
+T1595.002 - Vulnerability Scanning
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K6" s="3" t="n"/>
       <s:c r="L6" s="3" t="n"/>
       <s:c r="M6" s="3" t="n"/>
@@ -851,7 +872,14 @@
         </s:is>
       </s:c>
       <s:c r="I7" s="3" t="n"/>
-      <s:c r="J7" s="3" t="n"/>
+      <s:c r="J7" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1069.002 - Domain Groups
+T1482 - Domain Trust Discovery
+T1615 - Group Policy Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K7" s="3" t="n"/>
       <s:c r="L7" s="3" t="n"/>
       <s:c r="M7" s="3" t="n"/>
@@ -898,7 +926,14 @@
         </s:is>
       </s:c>
       <s:c r="I8" s="3" t="n"/>
-      <s:c r="J8" s="3" t="n"/>
+      <s:c r="J8" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1069.002 - Domain Groups
+T1482 - Domain Trust Discovery
+T1615 - Group Policy Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K8" s="3" t="n"/>
       <s:c r="L8" s="3" t="n"/>
       <s:c r="M8" s="3" t="n"/>
@@ -957,7 +992,12 @@
           <s:t>Get-ADUser -Filter {PasswordNotRequired -eq $true}</s:t>
         </s:is>
       </s:c>
-      <s:c r="J10" s="3" t="n"/>
+      <s:c r="J10" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1110 - Brute Force</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K10" s="3" t="n"/>
       <s:c r="L10" s="3" t="n"/>
       <s:c r="M10" s="3" t="n"/>
@@ -998,7 +1038,12 @@
           <s:t>Get-ADUser -Filter {PasswordNeverExpires -eq $true}</s:t>
         </s:is>
       </s:c>
-      <s:c r="J11" s="3" t="n"/>
+      <s:c r="J11" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1110.003 - Password Spraying</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K11" s="3" t="n"/>
       <s:c r="L11" s="3" t="n"/>
       <s:c r="M11" s="3" t="n"/>
@@ -1039,7 +1084,12 @@
           <s:t>Get-ADUser -Filter 'useraccountcontrol -band 4194304' -Properties useraccountcontrol | Format-Table name</s:t>
         </s:is>
       </s:c>
-      <s:c r="J12" s="3" t="n"/>
+      <s:c r="J12" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558.004 - AS-REP Roasting
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K12" s="3" t="n"/>
       <s:c r="L12" s="3" t="n"/>
       <s:c r="M12" s="3" t="n"/>
@@ -1083,7 +1133,13 @@
 Get-ADObject -SearchBase (Get-ADObject -Filter * -SearchBase (Get-ADDomain).DistinguishedName -SearchScope OneLevel).DistinguishedName -Filter 'adminCount -eq 1' -Properties adminCount</s:t>
         </s:is>
       </s:c>
-      <s:c r="J13" s="3" t="n"/>
+      <s:c r="J13" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1098 - Account Manipulation
+T1069.002 - Domain Groups</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K13" s="3" t="n"/>
       <s:c r="L13" s="3" t="n"/>
       <s:c r="M13" s="3" t="n"/>
@@ -1125,7 +1181,12 @@
 Get-ADComputer -Filter * -Properties primaryGroupID | Where-Object { $_.primaryGroupID -notin $defaults } | Select-Object Name, primaryGroupID</s:t>
         </s:is>
       </s:c>
-      <s:c r="J14" s="3" t="n"/>
+      <s:c r="J14" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1069.002 - Domain Groups</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K14" s="3" t="n"/>
       <s:c r="L14" s="3" t="n"/>
       <s:c r="M14" s="3" t="n"/>
@@ -1165,7 +1226,11 @@
 Get-ADComputer -Filter * -Properties primaryGroupID | Where-Object { -not $_.primaryGroupID } | Select-Object Name</s:t>
         </s:is>
       </s:c>
-      <s:c r="J15" s="3" t="n"/>
+      <s:c r="J15" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K15" s="3" t="n"/>
       <s:c r="L15" s="3" t="n"/>
       <s:c r="M15" s="3" t="n"/>
@@ -1207,7 +1272,12 @@
 # Review Default Domain Controllers Policy + tiering GPOs for Allow/Deny logon rights</s:t>
         </s:is>
       </s:c>
-      <s:c r="J16" s="3" t="n"/>
+      <s:c r="J16" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1021.002 - SMB/Windows Admin Shares</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K16" s="3" t="n"/>
       <s:c r="L16" s="3" t="n"/>
       <s:c r="M16" s="3" t="n"/>
@@ -1281,7 +1351,12 @@
 }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J17" s="3" t="n"/>
+      <s:c r="J17" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558.003 - Kerberoasting
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K17" s="3" t="n"/>
       <s:c r="L17" s="3" t="n"/>
       <s:c r="M17" s="3" t="n"/>
@@ -1322,7 +1397,12 @@
           <s:t>Get-ADUser -Filter 'servicePrincipalName -like "*"' -Properties servicePrincipalName, MemberOf | Select-Object Name, SamAccountName, servicePrincipalName, MemberOf</s:t>
         </s:is>
       </s:c>
-      <s:c r="J18" s="3" t="n"/>
+      <s:c r="J18" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558.003 - Kerberoasting
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K18" s="3" t="n"/>
       <s:c r="L18" s="3" t="n"/>
       <s:c r="M18" s="3" t="n"/>
@@ -1362,7 +1442,13 @@
 Get-GPO -All | Where-Object { $_.DisplayName -match 'DC|Domain Controller' } | ForEach-Object { gpresult /Scope Computer /Target $env:COMPUTERNAME /H "gpo-$($_.DisplayName).html" /F }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J19" s="3" t="n"/>
+      <s:c r="J19" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1021.002 - SMB/Windows Admin Shares
+T1021.001 - Remote Desktop Protocol</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K19" s="3" t="n"/>
       <s:c r="L19" s="3" t="n"/>
       <s:c r="M19" s="3" t="n"/>
@@ -1402,7 +1488,13 @@
 # Also review ACLs on SYSVOL\&lt;domain&gt;\scripts and GPO logon script deployment permissions</s:t>
         </s:is>
       </s:c>
-      <s:c r="J20" s="3" t="n"/>
+      <s:c r="J20" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1037.001 - Logon Script (Windows)
+T1098 - Account Manipulation
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K20" s="3" t="n"/>
       <s:c r="L20" s="3" t="n"/>
       <s:c r="M20" s="3" t="n"/>
@@ -1442,7 +1534,12 @@
           <s:t>Get-ADUser -Filter {SamAccountName -eq 'Guest'} -Properties Enabled, adminCount | Select-Object Name, Enabled</s:t>
         </s:is>
       </s:c>
-      <s:c r="J21" s="3" t="n"/>
+      <s:c r="J21" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.001 - Default Accounts
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K21" s="3" t="n"/>
       <s:c r="L21" s="3" t="n"/>
       <s:c r="M21" s="3" t="n"/>
@@ -1482,7 +1579,12 @@
 # Review ACLs on CN=Directory Service,CN=Windows NT,CN=Services,... and DPAPI-NG objects</s:t>
         </s:is>
       </s:c>
-      <s:c r="J22" s="3" t="n"/>
+      <s:c r="J22" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1555 - Credentials from Password Stores
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K22" s="3" t="n"/>
       <s:c r="L22" s="3" t="n"/>
       <s:c r="M22" s="3" t="n"/>
@@ -1524,7 +1626,12 @@
 Get-Acl "AD:\$domain" | Select-Object -ExpandProperty Access | Where-Object { $_.ActiveDirectoryRights -match 'Replicating Directory' } | Select-Object IdentityReference, ActiveDirectoryRights</s:t>
         </s:is>
       </s:c>
-      <s:c r="J23" s="3" t="n"/>
+      <s:c r="J23" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1003.006 - DCSync
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K23" s="3" t="n"/>
       <s:c r="L23" s="3" t="n"/>
       <s:c r="M23" s="3" t="n"/>
@@ -1563,7 +1670,12 @@
           <s:t>Get-Acl (Get-ADDomain).DistinguishedName | Select-Object -ExpandProperty Access | Where-Object { $_.ActiveDirectoryRights -match 'Validated-SPN|Self-Membership|WriteAccountRestrictions' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J24" s="3" t="n"/>
+      <s:c r="J24" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1136.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K24" s="3" t="n"/>
       <s:c r="L24" s="3" t="n"/>
       <s:c r="M24" s="3" t="n"/>
@@ -1602,7 +1714,12 @@
           <s:t>Get-WinEvent -FilterHashtable @{LogName='Security'; Id=4624} -MaxEvents 500 | Where-Object { $_.Properties[5].Value -match 'Administrator' -and $_.Properties[18].Value -match 'Logon Type:\\s*10|2' } | Select-Object TimeCreated, @{N='Account';E={$_.Properties[5].Value}} -First 20</s:t>
         </s:is>
       </s:c>
-      <s:c r="J25" s="3" t="n"/>
+      <s:c r="J25" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1078.001 - Default Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K25" s="3" t="n"/>
       <s:c r="L25" s="3" t="n"/>
       <s:c r="M25" s="3" t="n"/>
@@ -1641,7 +1758,12 @@
           <s:t>Get-ADUser -Filter 'altSecurityIdentities -like "*"' -Properties altSecurityIdentities | Select-Object Name, SamAccountName, altSecurityIdentities</s:t>
         </s:is>
       </s:c>
-      <s:c r="J26" s="3" t="n"/>
+      <s:c r="J26" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1556 - Modify Authentication Process</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K26" s="3" t="n"/>
       <s:c r="L26" s="3" t="n"/>
       <s:c r="M26" s="3" t="n"/>
@@ -1681,7 +1803,12 @@
 Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Services\Netlogon\Parameters' -Name RefusePasswordChange -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J27" s="3" t="n"/>
+      <s:c r="J27" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K27" s="3" t="n"/>
       <s:c r="L27" s="3" t="n"/>
       <s:c r="M27" s="3" t="n"/>
@@ -1720,7 +1847,12 @@
           <s:t>Get-ADGroupMember 'Domain Admins' -Recursive | Get-ADUser -Properties PasswordNeverExpires, servicePrincipalName | Where-Object { $_.PasswordNeverExpires -eq $true -or $_.servicePrincipalName } | Select-Object Name, SamAccountName, PasswordNeverExpires, servicePrincipalName</s:t>
         </s:is>
       </s:c>
-      <s:c r="J28" s="3" t="n"/>
+      <s:c r="J28" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K28" s="3" t="n"/>
       <s:c r="L28" s="3" t="n"/>
       <s:c r="M28" s="3" t="n"/>
@@ -1762,7 +1894,12 @@
 Get-ADObject -Filter 'objectClass -eq "domainDNS"' -Properties ms-DS-MachineAccountQuota | Select-Object ms-DS-MachineAccountQuota</s:t>
         </s:is>
       </s:c>
-      <s:c r="J29" s="3" t="n"/>
+      <s:c r="J29" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1136.002 - Domain Account
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K29" s="3" t="n"/>
       <s:c r="L29" s="3" t="n"/>
       <s:c r="M29" s="3" t="n"/>
@@ -1800,7 +1937,12 @@
 Get-ADComputer -Filter * -Properties primaryGroupID | Where-Object { $_.primaryGroupID -notin $defaults } | Select-Object Name, primaryGroupID</s:t>
         </s:is>
       </s:c>
-      <s:c r="J30" s="3" t="n"/>
+      <s:c r="J30" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1069.002 - Domain Groups</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K30" s="3" t="n"/>
       <s:c r="L30" s="3" t="n"/>
       <s:c r="M30" s="3" t="n"/>
@@ -1839,7 +1981,12 @@
           <s:t>Get-ADUser -Filter {SamAccountName -eq 'Administrator' -or SamAccountName -eq 'Guest'} | Select-Object Name, SamAccountName, Enabled</s:t>
         </s:is>
       </s:c>
-      <s:c r="J31" s="3" t="n"/>
+      <s:c r="J31" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.001 - Default Accounts
+T1036.005 - Match Legitimate Resource Name or Location</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K31" s="3" t="n"/>
       <s:c r="L31" s="3" t="n"/>
       <s:c r="M31" s="3" t="n"/>
@@ -1879,7 +2026,12 @@
 # Expect: duration &gt;=15m, threshold &lt;=5 (not 0), reset counter &gt;=15m</s:t>
         </s:is>
       </s:c>
-      <s:c r="J32" s="3" t="n"/>
+      <s:c r="J32" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1110 - Brute Force
+T1201 - Password Policy Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K32" s="3" t="n"/>
       <s:c r="L32" s="3" t="n"/>
       <s:c r="M32" s="3" t="n"/>
@@ -1937,7 +2089,12 @@
           <s:t>Get-ADGroupMember 'Domain Admins','Enterprise Admins','Schema Admins' -Recursive | Where-Object { $_.objectClass -eq 'computer' } | Select-Object Name, SamAccountName</s:t>
         </s:is>
       </s:c>
-      <s:c r="J34" s="3" t="n"/>
+      <s:c r="J34" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1069.002 - Domain Groups</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K34" s="3" t="n"/>
       <s:c r="L34" s="3" t="n"/>
       <s:c r="M34" s="3" t="n"/>
@@ -1978,7 +2135,12 @@
 Compare-Object (Get-ADGroupMember 'Domain Admins') (Get-ADGroupMember 'Protected Users' -ErrorAction SilentlyContinue) -Property Name -PassThru</s:t>
         </s:is>
       </s:c>
-      <s:c r="J35" s="3" t="n"/>
+      <s:c r="J35" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558 - Steal or Forge Kerberos Tickets
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K35" s="3" t="n"/>
       <s:c r="L35" s="3" t="n"/>
       <s:c r="M35" s="3" t="n"/>
@@ -2017,7 +2179,12 @@
           <s:t>Get-ADGroupMember 'Domain Admins','Enterprise Admins' | Where-Object { $_.Name -like '*ForeignSecurityPrincipals*' -or $_.SID -match 'S-1-5-21' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J36" s="3" t="n"/>
+      <s:c r="J36" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1482 - Domain Trust Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K36" s="3" t="n"/>
       <s:c r="L36" s="3" t="n"/>
       <s:c r="M36" s="3" t="n"/>
@@ -2057,7 +2224,12 @@
           <s:t>Get-ADGroupMember 'Account Operators','Server Operators','Backup Operators','Print Operators' | Select-Object Name, SamAccountName, objectClass</s:t>
         </s:is>
       </s:c>
-      <s:c r="J37" s="3" t="n"/>
+      <s:c r="J37" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1069.002 - Domain Groups
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K37" s="3" t="n"/>
       <s:c r="L37" s="3" t="n"/>
       <s:c r="M37" s="3" t="n"/>
@@ -2098,7 +2270,12 @@
 Get-ADUser -Filter * -Properties primaryGroupID | Where-Object { $_.primaryGroupID -notin 513,514,515,516,521 }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J38" s="3" t="n"/>
+      <s:c r="J38" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1069.002 - Domain Groups
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K38" s="3" t="n"/>
       <s:c r="L38" s="3" t="n"/>
       <s:c r="M38" s="3" t="n"/>
@@ -2137,7 +2314,12 @@
           <s:t>Get-ADGroup 'Protected Users' -ErrorAction SilentlyContinue | Select-Object Name, GroupScope, Members</s:t>
         </s:is>
       </s:c>
-      <s:c r="J39" s="3" t="n"/>
+      <s:c r="J39" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1069.002 - Domain Groups
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K39" s="3" t="n"/>
       <s:c r="L39" s="3" t="n"/>
       <s:c r="M39" s="3" t="n"/>
@@ -2179,7 +2361,12 @@
 Get-ADGroupMember 'Denied RODC Password Replication Group' | Select-Object Name</s:t>
         </s:is>
       </s:c>
-      <s:c r="J40" s="3" t="n"/>
+      <s:c r="J40" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1003.006 - DCSync
+T1484.002 - Trust Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K40" s="3" t="n"/>
       <s:c r="L40" s="3" t="n"/>
       <s:c r="M40" s="3" t="n"/>
@@ -2221,7 +2408,12 @@
           <s:t>Get-ADDomainController -Filter * | ForEach-Object { Get-ADObject $_.ComputerObjectDN -Properties msDS-RevealOnDemandGroup, msDS-NeverRevealGroup }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J41" s="3" t="n"/>
+      <s:c r="J41" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1069.002 - Domain Groups
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K41" s="3" t="n"/>
       <s:c r="L41" s="3" t="n"/>
       <s:c r="M41" s="3" t="n"/>
@@ -2264,7 +2456,12 @@
 # Should NOT include Authenticated Users; anonymous access must be disabled</s:t>
         </s:is>
       </s:c>
-      <s:c r="J42" s="3" t="n"/>
+      <s:c r="J42" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1550.002 - Pass the Hash</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K42" s="3" t="n"/>
       <s:c r="L42" s="3" t="n"/>
       <s:c r="M42" s="3" t="n"/>
@@ -2324,7 +2521,12 @@
 Get-ADGroupMember 'Domain Admins' | Select-Object Name, SamAccountName</s:t>
         </s:is>
       </s:c>
-      <s:c r="J44" s="3" t="n"/>
+      <s:c r="J44" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1069.002 - Domain Groups</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K44" s="3" t="n"/>
       <s:c r="L44" s="3" t="n"/>
       <s:c r="M44" s="3" t="n"/>
@@ -2363,7 +2565,12 @@
           <s:t>Get-ChildItem '\\$((Get-ADDomain).DNSRoot)\SYSVOL\$((Get-ADDomain).DNSRoot)\Policies' -Recurse -Filter 'DisplaySpecifier*' -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J45" s="3" t="n"/>
+      <s:c r="J45" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K45" s="3" t="n"/>
       <s:c r="L45" s="3" t="n"/>
       <s:c r="M45" s="3" t="n"/>
@@ -2398,7 +2605,12 @@
         </s:is>
       </s:c>
       <s:c r="I46" s="3" t="n"/>
-      <s:c r="J46" s="3" t="n"/>
+      <s:c r="J46" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1552.001 - Credentials In Files</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K46" s="3" t="n"/>
       <s:c r="L46" s="3" t="n"/>
       <s:c r="M46" s="3" t="n"/>
@@ -2443,7 +2655,12 @@
 Get-ADOrganizationalUnit -Filter * | ForEach-Object { Get-Acl "AD:\$($_.DistinguishedName)" | Select-Object -ExpandProperty Access | Where-Object { $_.IdentityReference -match 'Everyone|Authenticated Users|Domain Users' -and $_.ActiveDirectoryRights -match 'GenericAll|WriteDacl|WriteOwner' } }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J47" s="3" t="n"/>
+      <s:c r="J47" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K47" s="3" t="n"/>
       <s:c r="L47" s="3" t="n"/>
       <s:c r="M47" s="3" t="n"/>
@@ -2483,7 +2700,12 @@
           <s:t>Get-ChildItem "\\$((Get-ADDomain).DNSRoot)\SYSVOL" -Recurse | Get-Acl | Where-Object { $_.Access | Where-Object { $_.IdentityReference -match 'Everyone|Authenticated Users' -and $_.FileSystemRights -match 'Write|Modify|FullControl' } }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J48" s="3" t="n"/>
+      <s:c r="J48" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1484.001 - Group Policy Modification
+T1574.010 - Services File Permissions Weakness</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K48" s="3" t="n"/>
       <s:c r="L48" s="3" t="n"/>
       <s:c r="M48" s="3" t="n"/>
@@ -2528,7 +2750,12 @@
 (Get-ADObject "CN=Directory Service,CN=Windows NT,CN=Services,$cfg" -Properties dsHeuristics).dsHeuristics</s:t>
         </s:is>
       </s:c>
-      <s:c r="J49" s="3" t="n"/>
+      <s:c r="J49" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K49" s="3" t="n"/>
       <s:c r="L49" s="3" t="n"/>
       <s:c r="M49" s="3" t="n"/>
@@ -2568,7 +2795,12 @@
           <s:t>Get-ADDomainController -Filter * | ForEach-Object { Get-ADObject $_.ComputerObjectDN -Properties ManagedBy | Select-Object Name, ManagedBy }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J50" s="3" t="n"/>
+      <s:c r="J50" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K50" s="3" t="n"/>
       <s:c r="L50" s="3" t="n"/>
       <s:c r="M50" s="3" t="n"/>
@@ -2607,7 +2839,12 @@
           <s:t>Get-ADGroup 'Domain Admins','Enterprise Admins' | ForEach-Object { Get-ADObject $_.DistinguishedName -Properties ManagedBy | Select-Object Name, ManagedBy }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J51" s="3" t="n"/>
+      <s:c r="J51" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1222.001 - Windows Permissions</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K51" s="3" t="n"/>
       <s:c r="L51" s="3" t="n"/>
       <s:c r="M51" s="3" t="n"/>
@@ -2649,7 +2886,12 @@
 # 7th char of dsHeuristics != 0 may mask AdminSDHolder protection for some groups</s:t>
         </s:is>
       </s:c>
-      <s:c r="J52" s="3" t="n"/>
+      <s:c r="J52" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K52" s="3" t="n"/>
       <s:c r="L52" s="3" t="n"/>
       <s:c r="M52" s="3" t="n"/>
@@ -2689,7 +2931,12 @@
           <s:t>Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Services\LanmanServer\Parameters' -Name RestrictNullSessAccess, NullSessionPipes, NullSessionShares -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J53" s="3" t="n"/>
+      <s:c r="J53" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K53" s="3" t="n"/>
       <s:c r="L53" s="3" t="n"/>
       <s:c r="M53" s="3" t="n"/>
@@ -2733,7 +2980,12 @@
 auditpol /get /subcategory:'Account Logon'</s:t>
         </s:is>
       </s:c>
-      <s:c r="J54" s="3" t="n"/>
+      <s:c r="J54" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1562.002 - Disable Windows Event Logging
+T1070.001 - Clear Windows Event Logs</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K54" s="3" t="n"/>
       <s:c r="L54" s="3" t="n"/>
       <s:c r="M54" s="3" t="n"/>
@@ -2768,7 +3020,12 @@
         </s:is>
       </s:c>
       <s:c r="I55" s="3" t="n"/>
-      <s:c r="J55" s="3" t="n"/>
+      <s:c r="J55" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1059.001 - PowerShell
+T1562.002 - Disable Windows Event Logging</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K55" s="3" t="n"/>
       <s:c r="L55" s="3" t="n"/>
       <s:c r="M55" s="3" t="n"/>
@@ -2803,7 +3060,12 @@
         </s:is>
       </s:c>
       <s:c r="I56" s="3" t="n"/>
-      <s:c r="J56" s="3" t="n"/>
+      <s:c r="J56" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1021.002 - SMB/Windows Admin Shares
+T1187 - Forced Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K56" s="3" t="n"/>
       <s:c r="L56" s="3" t="n"/>
       <s:c r="M56" s="3" t="n"/>
@@ -2838,7 +3100,12 @@
         </s:is>
       </s:c>
       <s:c r="I57" s="3" t="n"/>
-      <s:c r="J57" s="3" t="n"/>
+      <s:c r="J57" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1557.001 - Name Resolution Poisoning and SMB Relay
+T1187 - Forced Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K57" s="3" t="n"/>
       <s:c r="L57" s="3" t="n"/>
       <s:c r="M57" s="3" t="n"/>
@@ -2879,7 +3146,12 @@
 dfsrmig /getmigrationstate</s:t>
         </s:is>
       </s:c>
-      <s:c r="J58" s="3" t="n"/>
+      <s:c r="J58" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1484.001 - Group Policy Modification
+T1570 - Lateral Tool Transfer</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K58" s="3" t="n"/>
       <s:c r="L58" s="3" t="n"/>
       <s:c r="M58" s="3" t="n"/>
@@ -2918,7 +3190,12 @@
           <s:t>Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Control\Lsa' -Name NoLMHash, LmCompatibilityLevel</s:t>
         </s:is>
       </s:c>
-      <s:c r="J59" s="3" t="n"/>
+      <s:c r="J59" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1110 - Brute Force
+T1556.005 - Reversible Encryption</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K59" s="3" t="n"/>
       <s:c r="L59" s="3" t="n"/>
       <s:c r="M59" s="3" t="n"/>
@@ -2966,7 +3243,12 @@
 Get-GPO -All | ForEach-Object { Get-GPOReport -Guid $_.Id -ReportType Xml | Select-String 'ClearTextPassword|ReversibleEncryption' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J60" s="3" t="n"/>
+      <s:c r="J60" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1552.001 - Credentials In Files
+T1552.006 - Group Policy Preferences</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K60" s="3" t="n"/>
       <s:c r="L60" s="3" t="n"/>
       <s:c r="M60" s="3" t="n"/>
@@ -3005,7 +3287,12 @@
           <s:t>Get-ADObject -SearchBase (Get-ADRootDSE).schemaNamingContext -Filter 'name -like "java*"' -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J61" s="3" t="n"/>
+      <s:c r="J61" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K61" s="3" t="n"/>
       <s:c r="L61" s="3" t="n"/>
       <s:c r="M61" s="3" t="n"/>
@@ -3050,7 +3337,12 @@
 Get-ADComputer -Filter 'sidHistory -like "*"' -Properties sidHistory | Select-Object Name, sidHistory</s:t>
         </s:is>
       </s:c>
-      <s:c r="J62" s="3" t="n"/>
+      <s:c r="J62" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K62" s="3" t="n"/>
       <s:c r="L62" s="3" t="n"/>
       <s:c r="M62" s="3" t="n"/>
@@ -3089,7 +3381,12 @@
           <s:t>Get-ADTrust -Filter * | Where-Object { $_.TrustType -eq 'Downlevel' } | Select-Object Name, Direction, TrustType, TrustAttributes</s:t>
         </s:is>
       </s:c>
-      <s:c r="J63" s="3" t="n"/>
+      <s:c r="J63" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1482 - Domain Trust Discovery
+T1484.002 - Trust Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K63" s="3" t="n"/>
       <s:c r="L63" s="3" t="n"/>
       <s:c r="M63" s="3" t="n"/>
@@ -3130,7 +3427,12 @@
           <s:t>Get-GPO -All | ForEach-Object { Get-GPOReport -Guid $_.Id -ReportType Html -Path "gpo-$($_.DisplayName).html" }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J64" s="3" t="n"/>
+      <s:c r="J64" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1484.001 - Group Policy Modification
+T1037.001 - Logon Script (Windows)</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K64" s="3" t="n"/>
       <s:c r="L64" s="3" t="n"/>
       <s:c r="M64" s="3" t="n"/>
@@ -3169,7 +3471,12 @@
           <s:t>Get-ADDomainController -Filter * | Select-Object Name, HostName, IPv4Address, IsGlobalCatalog, OperationMasterRoles</s:t>
         </s:is>
       </s:c>
-      <s:c r="J65" s="3" t="n"/>
+      <s:c r="J65" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K65" s="3" t="n"/>
       <s:c r="L65" s="3" t="n"/>
       <s:c r="M65" s="3" t="n"/>
@@ -3208,7 +3515,12 @@
           <s:t>Get-ADObject -SearchBase (Get-ADRootDSE).schemaNamingContext -Filter 'name -eq "computer"' -Properties mayContain</s:t>
         </s:is>
       </s:c>
-      <s:c r="J66" s="3" t="n"/>
+      <s:c r="J66" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098 - Account Manipulation
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K66" s="3" t="n"/>
       <s:c r="L66" s="3" t="n"/>
       <s:c r="M66" s="3" t="n"/>
@@ -3247,7 +3559,13 @@
           <s:t>Get-Acl "\\$((Get-ADDomain).DNSRoot)\SYSVOL" | Format-List</s:t>
         </s:is>
       </s:c>
-      <s:c r="J67" s="3" t="n"/>
+      <s:c r="J67" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1484.001 - Group Policy Modification
+T1574.010 - Services File Permissions Weakness
+T1037.001 - Logon Script (Windows)</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K67" s="3" t="n"/>
       <s:c r="L67" s="3" t="n"/>
       <s:c r="M67" s="3" t="n"/>
@@ -3282,7 +3600,12 @@
         </s:is>
       </s:c>
       <s:c r="I68" s="3" t="n"/>
-      <s:c r="J68" s="3" t="n"/>
+      <s:c r="J68" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1021.002 - SMB/Windows Admin Shares
+T1040 - Network Sniffing</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K68" s="3" t="n"/>
       <s:c r="L68" s="3" t="n"/>
       <s:c r="M68" s="3" t="n"/>
@@ -3321,7 +3644,12 @@
           <s:t>Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Services\LanmanServer\Parameters' -Name RestrictNullSessAccess, NullSessionPipes, NullSessionShares</s:t>
         </s:is>
       </s:c>
-      <s:c r="J69" s="3" t="n"/>
+      <s:c r="J69" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K69" s="3" t="n"/>
       <s:c r="L69" s="3" t="n"/>
       <s:c r="M69" s="3" t="n"/>
@@ -3360,7 +3688,12 @@
           <s:t>Get-ADTrust -Filter * | ForEach-Object { Get-ADTrust -Identity $_.Name -Properties sidFiltering, SelectiveAuthentication | Select-Object Name, Direction, sidFiltering, SelectiveAuthentication }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J70" s="3" t="n"/>
+      <s:c r="J70" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1482 - Domain Trust Discovery
+T1134 - Access Token Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K70" s="3" t="n"/>
       <s:c r="L70" s="3" t="n"/>
       <s:c r="M70" s="3" t="n"/>
@@ -3399,7 +3732,12 @@
           <s:t>Get-GPO -All | ForEach-Object { Get-GPOReport -Guid $_.Id -ReportType Xml | Select-String '\\.*\' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J71" s="3" t="n"/>
+      <s:c r="J71" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1570 - Lateral Tool Transfer
+T1021.002 - SMB/Windows Admin Shares</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K71" s="3" t="n"/>
       <s:c r="L71" s="3" t="n"/>
       <s:c r="M71" s="3" t="n"/>
@@ -3438,7 +3776,12 @@
           <s:t>Get-ADUser -Filter 'scriptPath -like "*"' -Properties scriptPath | Select-Object Name, scriptPath</s:t>
         </s:is>
       </s:c>
-      <s:c r="J72" s="3" t="n"/>
+      <s:c r="J72" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1037.003 - Network Logon Script
+T1570 - Lateral Tool Transfer</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K72" s="3" t="n"/>
       <s:c r="L72" s="3" t="n"/>
       <s:c r="M72" s="3" t="n"/>
@@ -3478,7 +3821,12 @@
 # Cross-reference last inter-domain auth in Security log (4769/4624)</s:t>
         </s:is>
       </s:c>
-      <s:c r="J73" s="3" t="n"/>
+      <s:c r="J73" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1482 - Domain Trust Discovery
+T1484.002 - Trust Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K73" s="3" t="n"/>
       <s:c r="L73" s="3" t="n"/>
       <s:c r="M73" s="3" t="n"/>
@@ -3520,7 +3868,12 @@
           <s:t>Get-ADDefaultDomainPasswordPolicy -Server Domainname</s:t>
         </s:is>
       </s:c>
-      <s:c r="J74" s="3" t="n"/>
+      <s:c r="J74" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1110 - Brute Force
+T1201 - Password Policy Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K74" s="3" t="n"/>
       <s:c r="L74" s="3" t="n"/>
       <s:c r="M74" s="3" t="n"/>
@@ -3559,7 +3912,12 @@
           <s:t>Get-GPO -All | ForEach-Object { Get-GPOReport -Guid $_.Id -ReportType Xml | Select-String 'RestrictSendingNTLM|RestrictReceivingNTLM|LmCompatibilityLevel' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J75" s="3" t="n"/>
+      <s:c r="J75" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1550.002 - Pass the Hash
+T1556.004 - Network Device Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K75" s="3" t="n"/>
       <s:c r="L75" s="3" t="n"/>
       <s:c r="M75" s="3" t="n"/>
@@ -3626,7 +3984,12 @@
 Get-DnsServerZoneTransfer -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J77" s="3" t="n"/>
+      <s:c r="J77" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1590.002 - DNS
+T1016 - System Network Configuration Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K77" s="3" t="n"/>
       <s:c r="L77" s="3" t="n"/>
       <s:c r="M77" s="3" t="n"/>
@@ -3667,7 +4030,12 @@
 certutil -caconfig -errorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J78" s="3" t="n"/>
+      <s:c r="J78" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1550.002 - Pass the Hash</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K78" s="3" t="n"/>
       <s:c r="L78" s="3" t="n"/>
       <s:c r="M78" s="3" t="n"/>
@@ -3709,7 +4077,12 @@
 Get-ADObject -SearchBase (Get-ADDomain).DistinguishedName -Filter 'objectClass -eq "msKds-ProvRootKey"'</s:t>
         </s:is>
       </s:c>
-      <s:c r="J79" s="3" t="n"/>
+      <s:c r="J79" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1552.006 - Group Policy Preferences
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K79" s="3" t="n"/>
       <s:c r="L79" s="3" t="n"/>
       <s:c r="M79" s="3" t="n"/>
@@ -3753,7 +4126,12 @@
 Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Services\NTDS\Parameters' -Name LdapEnforceChannelBinding, LDAPServerIntegrity -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J80" s="3" t="n"/>
+      <s:c r="J80" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1018 - Remote System Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K80" s="3" t="n"/>
       <s:c r="L80" s="3" t="n"/>
       <s:c r="M80" s="3" t="n"/>
@@ -3793,7 +4171,12 @@
 Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Control\Lsa\Kerberos\Parameters' -Name SupportedEncryptionTypes -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J81" s="3" t="n"/>
+      <s:c r="J81" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1600 - Weaken Encryption
+T1556.005 - Reversible Encryption</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K81" s="3" t="n"/>
       <s:c r="L81" s="3" t="n"/>
       <s:c r="M81" s="3" t="n"/>
@@ -3833,7 +4216,12 @@
           <s:t>Get-ItemProperty 'HKLM:\SYSTEM\CurrentControlSet\Services\Kdc' -Name EnableCbacAndArmor -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J82" s="3" t="n"/>
+      <s:c r="J82" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558 - Steal or Forge Kerberos Tickets
+T1556.004 - Network Device Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K82" s="3" t="n"/>
       <s:c r="L82" s="3" t="n"/>
       <s:c r="M82" s="3" t="n"/>
@@ -3877,7 +4265,12 @@
 Get-ADObject -Filter 'msDS-SupportedEncryptionTypes -like "*"' -Properties msDS-SupportedEncryptionTypes -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J83" s="3" t="n"/>
+      <s:c r="J83" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1558 - Steal or Forge Kerberos Tickets
+T1550.003 - Pass the Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K83" s="3" t="n"/>
       <s:c r="L83" s="3" t="n"/>
       <s:c r="M83" s="3" t="n"/>
@@ -3915,7 +4308,12 @@
         </s:is>
       </s:c>
       <s:c r="I84" s="3" t="n"/>
-      <s:c r="J84" s="3" t="n"/>
+      <s:c r="J84" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1021.002 - SMB/Windows Admin Shares
+T1557.001 - Name Resolution Poisoning and SMB Relay</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K84" s="3" t="n"/>
       <s:c r="L84" s="3" t="n"/>
       <s:c r="M84" s="3" t="n"/>
@@ -3951,7 +4349,12 @@
         </s:is>
       </s:c>
       <s:c r="I85" s="3" t="n"/>
-      <s:c r="J85" s="3" t="n"/>
+      <s:c r="J85" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1210 - Exploitation of Remote Services
+T1489 - Service Stop</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K85" s="3" t="n"/>
       <s:c r="L85" s="3" t="n"/>
       <s:c r="M85" s="3" t="n"/>
@@ -3994,7 +4397,12 @@
 Get-ChildItem 'HKLM:\SOFTWARE\Microsoft\Windows\CurrentVersion\Policies\LAPS' -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J86" s="3" t="n"/>
+      <s:c r="J86" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1552.001 - Credentials In Files</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K86" s="3" t="n"/>
       <s:c r="L86" s="3" t="n"/>
       <s:c r="M86" s="3" t="n"/>
@@ -4029,7 +4437,12 @@
         </s:is>
       </s:c>
       <s:c r="I87" s="3" t="n"/>
-      <s:c r="J87" s="3" t="n"/>
+      <s:c r="J87" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1187 - Forced Authentication
+T1210 - Exploitation of Remote Services</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K87" s="3" t="n"/>
       <s:c r="L87" s="3" t="n"/>
       <s:c r="M87" s="3" t="n"/>
@@ -4067,7 +4480,12 @@
         </s:is>
       </s:c>
       <s:c r="I88" s="3" t="n"/>
-      <s:c r="J88" s="3" t="n"/>
+      <s:c r="J88" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1072 - Software Deployment Tools
+T1195.002 - Compromise Software Supply Chain</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K88" s="3" t="n"/>
       <s:c r="L88" s="3" t="n"/>
       <s:c r="M88" s="3" t="n"/>
@@ -4125,7 +4543,13 @@
           <s:t>Get-ADUser -Filter 'Description -like "*Azure*AD*Connect*"' -Properties PasswordLastSet, Enabled | Select-Object Name, PasswordLastSet, Enabled</s:t>
         </s:is>
       </s:c>
-      <s:c r="J90" s="3" t="n"/>
+      <s:c r="J90" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1556.007 - Hybrid Identity
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K90" s="3" t="n"/>
       <s:c r="L90" s="3" t="n"/>
       <s:c r="M90" s="3" t="n"/>
@@ -4165,7 +4589,12 @@
 # Cross-reference with Entra ID synced users (Graph / AzureAD module)</s:t>
         </s:is>
       </s:c>
-      <s:c r="J91" s="3" t="n"/>
+      <s:c r="J91" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K91" s="3" t="n"/>
       <s:c r="L91" s="3" t="n"/>
       <s:c r="M91" s="3" t="n"/>
@@ -4205,7 +4634,12 @@
 Get-MgIdentityConditionalAccessPolicy | Where-Object { $_.SessionControls.SignInFrequency.IsEnabled -eq $false } | Select-Object DisplayName</s:t>
         </s:is>
       </s:c>
-      <s:c r="J92" s="3" t="n"/>
+      <s:c r="J92" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K92" s="3" t="n"/>
       <s:c r="L92" s="3" t="n"/>
       <s:c r="M92" s="3" t="n"/>
@@ -4245,7 +4679,12 @@
 (Get-MgDirectoryAdministrativeUnit -All).Count</s:t>
         </s:is>
       </s:c>
-      <s:c r="J93" s="3" t="n"/>
+      <s:c r="J93" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098.003 - Additional Cloud Roles
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K93" s="3" t="n"/>
       <s:c r="L93" s="3" t="n"/>
       <s:c r="M93" s="3" t="n"/>
@@ -4285,7 +4724,12 @@
 # Cross-reference with Entra privileged role members (Graph / AzureAD module)</s:t>
         </s:is>
       </s:c>
-      <s:c r="J94" s="3" t="n"/>
+      <s:c r="J94" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K94" s="3" t="n"/>
       <s:c r="L94" s="3" t="n"/>
       <s:c r="M94" s="3" t="n"/>
@@ -4325,7 +4769,12 @@
 Get-MgPolicyAuthorizationPolicy | Select-Object -ExpandProperty DefaultUserRolePermissions</s:t>
         </s:is>
       </s:c>
-      <s:c r="J95" s="3" t="n"/>
+      <s:c r="J95" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098.003 - Additional Cloud Roles
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K95" s="3" t="n"/>
       <s:c r="L95" s="3" t="n"/>
       <s:c r="M95" s="3" t="n"/>
@@ -4365,7 +4814,12 @@
           <s:t>Get-ADUser -Filter 'DisplayName -like "*AZUREADSSO*"' -Properties PasswordLastSet | Select-Object Name, PasswordLastSet</s:t>
         </s:is>
       </s:c>
-      <s:c r="J96" s="3" t="n"/>
+      <s:c r="J96" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1556.007 - Hybrid Identity
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K96" s="3" t="n"/>
       <s:c r="L96" s="3" t="n"/>
       <s:c r="M96" s="3" t="n"/>
@@ -4405,7 +4859,12 @@
 Get-MgIdentityConditionalAccessPolicy | Select-Object DisplayName, SessionControls</s:t>
         </s:is>
       </s:c>
-      <s:c r="J97" s="3" t="n"/>
+      <s:c r="J97" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1556.009 - Conditional Access Policies
+T1078.004 - Cloud Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K97" s="3" t="n"/>
       <s:c r="L97" s="3" t="n"/>
       <s:c r="M97" s="3" t="n"/>
@@ -4445,7 +4904,12 @@
 Get-MgDirectoryRoleMember -DirectoryRoleId (Get-MgDirectoryRole -Filter "displayName eq 'Global Administrator'").Id</s:t>
         </s:is>
       </s:c>
-      <s:c r="J98" s="3" t="n"/>
+      <s:c r="J98" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K98" s="3" t="n"/>
       <s:c r="L98" s="3" t="n"/>
       <s:c r="M98" s="3" t="n"/>
@@ -4485,7 +4949,12 @@
 (Get-MgPolicyAuthorizationPolicy).DefaultUserRolePermissions | Select-Object AllowedToCreateApps</s:t>
         </s:is>
       </s:c>
-      <s:c r="J99" s="3" t="n"/>
+      <s:c r="J99" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1098.003 - Additional Cloud Roles
+T1528 - Steal Application Access Token</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K99" s="3" t="n"/>
       <s:c r="L99" s="3" t="n"/>
       <s:c r="M99" s="3" t="n"/>
@@ -4525,7 +4994,12 @@
 Get-MgRoleManagementDirectoryRoleAssignment -ExpandProperty Principal</s:t>
         </s:is>
       </s:c>
-      <s:c r="J100" s="3" t="n"/>
+      <s:c r="J100" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K100" s="3" t="n"/>
       <s:c r="L100" s="3" t="n"/>
       <s:c r="M100" s="3" t="n"/>
@@ -4566,7 +5040,12 @@
 Get-MgUser -Filter "userType eq 'Guest'" -All | Select-Object DisplayName, UserPrincipalName</s:t>
         </s:is>
       </s:c>
-      <s:c r="J101" s="3" t="n"/>
+      <s:c r="J101" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K101" s="3" t="n"/>
       <s:c r="L101" s="3" t="n"/>
       <s:c r="M101" s="3" t="n"/>
@@ -4606,7 +5085,12 @@
 Get-MgPolicyAuthorizationPolicy | Select-Object -ExpandProperty DefaultUserRolePermissions</s:t>
         </s:is>
       </s:c>
-      <s:c r="J102" s="3" t="n"/>
+      <s:c r="J102" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1528 - Steal Application Access Token
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K102" s="3" t="n"/>
       <s:c r="L102" s="3" t="n"/>
       <s:c r="M102" s="3" t="n"/>
@@ -4646,7 +5130,12 @@
 Get-MgIdentityConditionalAccessPolicy | Where-Object { $_.Conditions.SignInRiskLevels }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J103" s="3" t="n"/>
+      <s:c r="J103" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1110.003 - Password Spraying</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K103" s="3" t="n"/>
       <s:c r="L103" s="3" t="n"/>
       <s:c r="M103" s="3" t="n"/>
@@ -4686,7 +5175,12 @@
 Get-MgServicePrincipal -All | ForEach-Object { Get-MgServicePrincipalAppRoleAssignedTo -ServicePrincipalId $_.Id }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J104" s="3" t="n"/>
+      <s:c r="J104" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1528 - Steal Application Access Token
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K104" s="3" t="n"/>
       <s:c r="L104" s="3" t="n"/>
       <s:c r="M104" s="3" t="n"/>
@@ -4726,7 +5220,12 @@
 Get-MgIdentityConditionalAccessPolicy | Select-Object DisplayName, Conditions</s:t>
         </s:is>
       </s:c>
-      <s:c r="J105" s="3" t="n"/>
+      <s:c r="J105" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1556.006 - Multi-Factor Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K105" s="3" t="n"/>
       <s:c r="L105" s="3" t="n"/>
       <s:c r="M105" s="3" t="n"/>
@@ -4767,7 +5266,12 @@
 # REVIEW if Conditional Access replaces Security Defaults</s:t>
         </s:is>
       </s:c>
-      <s:c r="J106" s="3" t="n"/>
+      <s:c r="J106" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1556.006 - Multi-Factor Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K106" s="3" t="n"/>
       <s:c r="L106" s="3" t="n"/>
       <s:c r="M106" s="3" t="n"/>
@@ -4807,7 +5311,12 @@
 Get-MgUser -Filter "userType eq 'Guest' and externalUserState eq 'PendingAcceptance'" -All</s:t>
         </s:is>
       </s:c>
-      <s:c r="J107" s="3" t="n"/>
+      <s:c r="J107" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.004 - Cloud Accounts
+T1098.003 - Additional Cloud Roles</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K107" s="3" t="n"/>
       <s:c r="L107" s="3" t="n"/>
       <s:c r="M107" s="3" t="n"/>
@@ -4849,7 +5358,12 @@
 Get-MgReportAuthenticationMethodUserRegistrationDetail -All | Where-Object { $_.IsMfaRegistered -eq $false -and $_.IsAdmin -eq $true }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J108" s="3" t="n"/>
+      <s:c r="J108" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1556.006 - Multi-Factor Authentication
+T1621 - Multi-Factor Authentication Request Generation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K108" s="3" t="n"/>
       <s:c r="L108" s="3" t="n"/>
       <s:c r="M108" s="3" t="n"/>
@@ -4888,7 +5402,12 @@
           <s:t>Get-ADObject -Filter 'msLAPS-PasswordExpirationTime -like "*"' -ErrorAction SilentlyContinue | Measure-Object | Select-Object Count</s:t>
         </s:is>
       </s:c>
-      <s:c r="J109" s="3" t="n"/>
+      <s:c r="J109" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1552.001 - Credentials In Files
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K109" s="3" t="n"/>
       <s:c r="L109" s="3" t="n"/>
       <s:c r="M109" s="3" t="n"/>
@@ -4946,7 +5465,12 @@
           <s:t>Get-ADUser -Filter {SamAccountName -eq 'Administrator'} -Properties TrustedForDelegation, TrustedToAuthForDelegation | Select-Object Name, TrustedForDelegation, TrustedToAuthForDelegation</s:t>
         </s:is>
       </s:c>
-      <s:c r="J111" s="3" t="n"/>
+      <s:c r="J111" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1558.001 - Golden Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K111" s="3" t="n"/>
       <s:c r="L111" s="3" t="n"/>
       <s:c r="M111" s="3" t="n"/>
@@ -4986,7 +5510,12 @@
 # Use BloodHound / Find-InterestingDomainAcl for Everyone/Authenticated Users delegations</s:t>
         </s:is>
       </s:c>
-      <s:c r="J112" s="3" t="n"/>
+      <s:c r="J112" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1558.001 - Golden Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K112" s="3" t="n"/>
       <s:c r="L112" s="3" t="n"/>
       <s:c r="M112" s="3" t="n"/>
@@ -5025,7 +5554,12 @@
           <s:t>Get-ADObject -Filter 'msDS-AllowedToActOnBehalfOfOtherIdentity -like "*"' -Properties msDS-AllowedToActOnBehalfOfOtherIdentity -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J113" s="3" t="n"/>
+      <s:c r="J113" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K113" s="3" t="n"/>
       <s:c r="L113" s="3" t="n"/>
       <s:c r="M113" s="3" t="n"/>
@@ -5067,7 +5601,12 @@
 Get-ADComputer -LDAPFilter "(userAccountControl:1.2.840.113556.1.4.803:=524288)"</s:t>
         </s:is>
       </s:c>
-      <s:c r="J114" s="3" t="n"/>
+      <s:c r="J114" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134.001 - Token Impersonation/Theft
+T1550.003 - Pass the Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K114" s="3" t="n"/>
       <s:c r="L114" s="3" t="n"/>
       <s:c r="M114" s="3" t="n"/>
@@ -5108,7 +5647,12 @@
           <s:t>Get-GPO -All | ForEach-Object { Get-GPPermission -Guid $_.Id -All | Where-Object { $_.Permission -eq 'GpoEdit' -or $_.Permission -eq 'GpoApply' } }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J115" s="3" t="n"/>
+      <s:c r="J115" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1484.001 - Group Policy Modification
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K115" s="3" t="n"/>
       <s:c r="L115" s="3" t="n"/>
       <s:c r="M115" s="3" t="n"/>
@@ -5150,7 +5694,12 @@
           <s:t>Get-ADComputer -Filter {TrustedToAuthForDelegation -eq $True -or msDS-AllowedToDelegateTo -like '*'} -Properties msDS-AllowedToDelegateTo, msDS-AllowedToActOnBehalfOfOtherIdentity | Where-Object { $_.Name -match 'DC' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J116" s="3" t="n"/>
+      <s:c r="J116" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1558.001 - Golden Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K116" s="3" t="n"/>
       <s:c r="L116" s="3" t="n"/>
       <s:c r="M116" s="3" t="n"/>
@@ -5197,7 +5746,12 @@
           <s:t>Get-ADObject -Filter 'msDS-AllowedToDelegateTo -like "*"' -Properties msDS-AllowedToDelegateTo, msDS-AllowedToActOnBehalfOfOtherIdentity | Select-Object Name, msDS-AllowedToDelegateTo</s:t>
         </s:is>
       </s:c>
-      <s:c r="J117" s="3" t="n"/>
+      <s:c r="J117" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1558.001 - Golden Ticket</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K117" s="3" t="n"/>
       <s:c r="L117" s="3" t="n"/>
       <s:c r="M117" s="3" t="n"/>
@@ -5238,7 +5792,13 @@
 # TrustAttributes 0x800 = TGT delegation (Selective Authentication should be enabled)</s:t>
         </s:is>
       </s:c>
-      <s:c r="J118" s="3" t="n"/>
+      <s:c r="J118" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1134 - Access Token Manipulation
+T1558.001 - Golden Ticket
+T1482 - Domain Trust Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K118" s="3" t="n"/>
       <s:c r="L118" s="3" t="n"/>
       <s:c r="M118" s="3" t="n"/>
@@ -5296,7 +5856,12 @@
           <s:t>certutil -template -v | Select-String 'CT_FLAG_ENROLLEE_SUPPLIES_SUBJECT|Supply in request'</s:t>
         </s:is>
       </s:c>
-      <s:c r="J120" s="3" t="n"/>
+      <s:c r="J120" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1553.004 - Install Root Certificate</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K120" s="3" t="n"/>
       <s:c r="L120" s="3" t="n"/>
       <s:c r="M120" s="3" t="n"/>
@@ -5340,7 +5905,12 @@
 Get-Acl 'CN=Certificate Templates,CN=Public Key Services,CN=Services,(Get-ADRootDSE).configurationNamingContext'</s:t>
         </s:is>
       </s:c>
-      <s:c r="J121" s="3" t="n"/>
+      <s:c r="J121" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K121" s="3" t="n"/>
       <s:c r="L121" s="3" t="n"/>
       <s:c r="M121" s="3" t="n"/>
@@ -5380,7 +5950,12 @@
 Get-Website | Where-Object { $_.Name -match 'CertSrv' }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J122" s="3" t="n"/>
+      <s:c r="J122" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1048.003 - Exfiltration Over Unencrypted Non-C2 Protocol</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K122" s="3" t="n"/>
       <s:c r="L122" s="3" t="n"/>
       <s:c r="M122" s="3" t="n"/>
@@ -5420,7 +5995,12 @@
           <s:t>certutil -template -v | Select-String 'Enrollment Permissions|Authenticated Users|Everyone|Domain Users'</s:t>
         </s:is>
       </s:c>
-      <s:c r="J123" s="3" t="n"/>
+      <s:c r="J123" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K123" s="3" t="n"/>
       <s:c r="L123" s="3" t="n"/>
       <s:c r="M123" s="3" t="n"/>
@@ -5459,7 +6039,12 @@
           <s:t>Get-WebConfigurationProperty -pspath 'MACHINE/WEBROOT/APPHOST' -filter "system.webServer/security/authentication/extendedProtection" -name enabled -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J124" s="3" t="n"/>
+      <s:c r="J124" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1187 - Forced Authentication</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K124" s="3" t="n"/>
       <s:c r="L124" s="3" t="n"/>
       <s:c r="M124" s="3" t="n"/>
@@ -5514,7 +6099,12 @@
 certutil -store CA</s:t>
         </s:is>
       </s:c>
-      <s:c r="J125" s="3" t="n"/>
+      <s:c r="J125" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1649 - Steal or Forge Authentication Certificates
+T1553.004 - Install Root Certificate</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K125" s="3" t="n"/>
       <s:c r="L125" s="3" t="n"/>
       <s:c r="M125" s="3" t="n"/>
@@ -5585,7 +6175,12 @@
 Get-ADUser -Filter {SamAccountName -eq 'krbtgt'} -Properties PasswordLastSet</s:t>
         </s:is>
       </s:c>
-      <s:c r="J127" s="3" t="n"/>
+      <s:c r="J127" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1110.003 - Password Spraying
+T1201 - Password Policy Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K127" s="3" t="n"/>
       <s:c r="L127" s="3" t="n"/>
       <s:c r="M127" s="3" t="n"/>
@@ -5627,7 +6222,12 @@
 Get-ADObject -Filter 'name -like "Exchange*"' -SearchBase (Get-ADDomain).DistinguishedName -ErrorAction SilentlyContinue</s:t>
         </s:is>
       </s:c>
-      <s:c r="J128" s="3" t="n"/>
+      <s:c r="J128" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1552.001 - Credentials In Files
+T1083 - File and Directory Discovery</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K128" s="3" t="n"/>
       <s:c r="L128" s="3" t="n"/>
       <s:c r="M128" s="3" t="n"/>
@@ -5668,7 +6268,12 @@
 Write-Output “Active Directory’s Tombstone Lifetime is set to $TombstoneLifetime days `r “</s:t>
         </s:is>
       </s:c>
-      <s:c r="J129" s="3" t="n"/>
+      <s:c r="J129" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1484.001 - Group Policy Modification</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K129" s="3" t="n"/>
       <s:c r="L129" s="3" t="n"/>
       <s:c r="M129" s="3" t="n"/>
@@ -5708,7 +6313,12 @@
 repadmin /showbackup</s:t>
         </s:is>
       </s:c>
-      <s:c r="J130" s="3" t="n"/>
+      <s:c r="J130" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1490 - Inhibit System Recovery
+T1485 - Data Destruction</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K130" s="3" t="n"/>
       <s:c r="L130" s="3" t="n"/>
       <s:c r="M130" s="3" t="n"/>
@@ -5748,7 +6358,12 @@
 Get-ADDomainController -Filter * | Select-Object Name, Site, IsGlobalCatalog, OperationMasterRoles</s:t>
         </s:is>
       </s:c>
-      <s:c r="J131" s="3" t="n"/>
+      <s:c r="J131" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1498 - Network Denial of Service
+T1486 - Data Encrypted for Impact</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K131" s="3" t="n"/>
       <s:c r="L131" s="3" t="n"/>
       <s:c r="M131" s="3" t="n"/>
@@ -5794,7 +6409,12 @@
 Search-ADAccount -AccountInactive -TimeSpan 90 -UsersOnly -ComputersOnly</s:t>
         </s:is>
       </s:c>
-      <s:c r="J132" s="3" t="n"/>
+      <s:c r="J132" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1087.002 - Domain Account
+T1078.002 - Domain Accounts</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K132" s="3" t="n"/>
       <s:c r="L132" s="3" t="n"/>
       <s:c r="M132" s="3" t="n"/>
@@ -5833,7 +6453,12 @@
           <s:t>Get-ADOptionalFeature -Filter 'Name -like "*Recycle*"' | Select-Object Name, EnabledScopes</s:t>
         </s:is>
       </s:c>
-      <s:c r="J133" s="3" t="n"/>
+      <s:c r="J133" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1485 - Data Destruction
+T1070 - Indicator Removal</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K133" s="3" t="n"/>
       <s:c r="L133" s="3" t="n"/>
       <s:c r="M133" s="3" t="n"/>
@@ -5874,7 +6499,12 @@
 (Get-ADGroupMember 'Schema Admins').Count</s:t>
         </s:is>
       </s:c>
-      <s:c r="J134" s="3" t="n"/>
+      <s:c r="J134" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1098 - Account Manipulation</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K134" s="3" t="n"/>
       <s:c r="L134" s="3" t="n"/>
       <s:c r="M134" s="3" t="n"/>
@@ -5917,7 +6547,12 @@
 Get-ADDomain | Select-Object Name, DomainMode</s:t>
         </s:is>
       </s:c>
-      <s:c r="J135" s="3" t="n"/>
+      <s:c r="J135" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1068 - Exploitation for Privilege Escalation
+T1190 - Exploit Public-Facing Application</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K135" s="3" t="n"/>
       <s:c r="L135" s="3" t="n"/>
       <s:c r="M135" s="3" t="n"/>
@@ -5964,7 +6599,12 @@
         </s:is>
       </s:c>
       <s:c r="I136" s="3" t="n"/>
-      <s:c r="J136" s="3" t="n"/>
+      <s:c r="J136" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1068 - Exploitation for Privilege Escalation
+T1190 - Exploit Public-Facing Application</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K136" s="3" t="n"/>
       <s:c r="L136" s="3" t="n"/>
       <s:c r="M136" s="3" t="n"/>
@@ -6003,7 +6643,12 @@
           <s:t>Get-ADUser -Filter * -Properties SamAccountName | Group-Object SamAccountName | Where-Object { $_.Count -gt 1 }</s:t>
         </s:is>
       </s:c>
-      <s:c r="J137" s="3" t="n"/>
+      <s:c r="J137" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1078.002 - Domain Accounts
+T1087.002 - Domain Account</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K137" s="3" t="n"/>
       <s:c r="L137" s="3" t="n"/>
       <s:c r="M137" s="3" t="n"/>
@@ -6038,7 +6683,12 @@
         </s:is>
       </s:c>
       <s:c r="I138" s="3" t="n"/>
-      <s:c r="J138" s="3" t="n"/>
+      <s:c r="J138" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1068 - Exploitation for Privilege Escalation
+T1190 - Exploit Public-Facing Application</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K138" s="3" t="n"/>
       <s:c r="L138" s="3" t="n"/>
       <s:c r="M138" s="3" t="n"/>
@@ -6075,7 +6725,12 @@
         </s:is>
       </s:c>
       <s:c r="I139" s="3" t="n"/>
-      <s:c r="J139" s="3" t="n"/>
+      <s:c r="J139" s="3" t="inlineStr">
+        <s:is>
+          <s:t>T1068 - Exploitation for Privilege Escalation
+T1190 - Exploit Public-Facing Application</s:t>
+        </s:is>
+      </s:c>
       <s:c r="K139" s="3" t="n"/>
       <s:c r="L139" s="3" t="n"/>
       <s:c r="M139" s="3" t="n"/>

</xml_diff>